<commit_message>
feat: TopSheet template v3 — 23 tabs, complete database coverage
Added missing tabs:
- 13. Holdings — account-level deal holdings
- 13B. Investors — external investor allocations per tranche
- 13C. Intercreditor — ICA terms, standstill, turnover, non-petition
- 13D. Enforcement Classes — multi-class covenant groupings

Added missing Deal Identity fields:
- Change of Control (regime, definition, consequence, prepayment basis)
- Equity Cure (available, regime description)
- Model Version and Date

23 tabs total. Auto-derivable tables (covenants, financial_periods,
deal_line_item_labels, forecast_cases, deal_obligation_register) are
generated by the ingestion engine and not needed in the template.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/topsheet-data-template-v3.xlsx
+++ b/docs/topsheet-data-template-v3.xlsx
@@ -20,12 +20,16 @@
     <sheet name="11. Development Phases" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="12. Consent Mechanics" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Validation" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="13. Period Definition" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="14. Management Case" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="15. Credit Case" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="16. Combined Downside" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="17. Actuals" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="18. Key Risks" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="13. Holdings" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="13B. Investors" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="13C. Intercreditor" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="13D. Enforcement Classes" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="14. Period Definition" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="15. Management Case" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="16. Credit Case" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="17. Combined Downside" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="18. Actuals" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="19. Key Risks" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -598,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1467,7 +1471,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>MONITORING</t>
+          <t>CHANGE OF CONTROL</t>
         </is>
       </c>
       <c r="B80" s="5" t="n"/>
@@ -1476,99 +1480,221 @@
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>Assigned HAM</t>
+          <t>CoC Regime Exists</t>
         </is>
       </c>
       <c r="B81" s="7" t="n"/>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Human Asset Manager</t>
+          <t>Yes/No</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>Assigned PM</t>
+          <t>CoC Definition</t>
         </is>
       </c>
       <c r="B82" s="7" t="n"/>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Portfolio Manager</t>
+          <t>How is 'control' defined?</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>Performance Grade</t>
-        </is>
-      </c>
-      <c r="B83" s="10" t="inlineStr">
-        <is>
-          <t>(computed)</t>
-        </is>
-      </c>
+          <t>CoC Consequence</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="n"/>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Computed by grade engine (1-4)</t>
+          <t>Mandatory prepayment, EoD, consent required</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
+          <t>CoC Prepayment Basis</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="n"/>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>par, make_whole, market_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>EQUITY CURE &amp; MODEL</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n"/>
+      <c r="C86" s="5" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>Equity Cure Available</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Yes/No</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>Equity Cure Regime</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="n"/>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Max frequency, amount limits, mechanism</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>Model Version</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="n"/>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>e.g. v3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>Model Date</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="n"/>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>MONITORING</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="n"/>
+      <c r="C92" s="5" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>Assigned HAM</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="n"/>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>Human Asset Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Assigned PM</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="n"/>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Portfolio Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>Performance Grade</t>
+        </is>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>(computed)</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Computed by grade engine (1-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
           <t>Watchlist</t>
         </is>
       </c>
-      <c r="B84" s="10" t="inlineStr">
+      <c r="B96" s="10" t="inlineStr">
         <is>
           <t>(computed)</t>
         </is>
       </c>
-      <c r="C84" s="8" t="inlineStr">
+      <c r="C96" s="8" t="inlineStr">
         <is>
           <t>Computed by grade engine</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="9" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="9" t="inlineStr">
         <is>
           <t>Trend</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B97" s="10" t="inlineStr">
         <is>
           <t>(computed)</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
+      <c r="C97" s="8" t="inlineStr">
         <is>
           <t>Computed from 3-period erosion</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="9" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="9" t="inlineStr">
         <is>
           <t>Headroom %</t>
         </is>
       </c>
-      <c r="B86" s="10" t="inlineStr">
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>(computed)</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr">
+      <c r="C98" s="8" t="inlineStr">
         <is>
           <t>Computed: (actual-default)/(mgmt-default) x 100</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A1:C1"/>
@@ -1577,12 +1703,14 @@
     <mergeCell ref="A61:C61"/>
     <mergeCell ref="A70:C70"/>
     <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A92:C92"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A86:C86"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Wind Farm,Data Center,Port,Airport,Toll Road,Social Infrastructure,Real Estate,Clean Tech Hub,Solar"</formula1>
     </dataValidation>
@@ -1597,6 +1725,12 @@
     </dataValidation>
     <dataValidation sqref="B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"very_low,low,moderate,high,very_high"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2359,13 +2493,13 @@
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"by_commitment,by_lender,by_block"</formula1>
     </dataValidation>
-    <dataValidation sqref="B7 B8 B9 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="B7 B8 B9 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="B7 B8 B9 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2594,6 +2728,521 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HOLDINGS — Which accounts hold this deal and how much</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Account Name</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Holding Amount</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Instrument Name</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Tranche Amount</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Acquisition Date</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Acquisition Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n"/>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INVESTOR ALLOCATIONS — External investors and their mandates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Investor Name</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Account / Mandate</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Tranche</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Mandate Size</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>% of Mandate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n"/>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INTERCREDITOR TERMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Provision</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Agreement Type</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>ICA, STID, Common Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Governing Law</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>English, New York, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement Standstill (days)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>e.g. 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Non-Petition Clause</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Yes/No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Turnover Provisions</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Permitted Payments</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Release Conditions</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Subrogation Rights</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ENFORCEMENT CLASSES — For multi-class capital structures (WBS, bond structures)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Class Code</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Included Instruments</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Distribution Conditions</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n"/>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3388,7 +4037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10388,7 +11037,306 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CAPITAL STRUCTURE INSTRUMENTS — One row per debt instrument</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Instrument Name</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Security Ranking</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Pari-Passu Group</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Committed Amount</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Drawn Amount</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Margin (bps)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Base Rate</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Interest Type</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Maturity Date</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Repayment Type</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Our Holding Amount</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Our Holding %</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>DSRA Months</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n"/>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
+      <c r="J3" s="7" t="n"/>
+      <c r="K3" s="7" t="n"/>
+      <c r="L3" s="7" t="n"/>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="7" t="n"/>
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="7" t="n"/>
+      <c r="Q3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="7" t="n"/>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="7" t="n"/>
+      <c r="Q4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="7" t="n"/>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
+      <c r="Q5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="7" t="n"/>
+      <c r="Q6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
+      <c r="Q7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
+      <c r="Q9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
+      <c r="Q10" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:Q1"/>
+  </mergeCells>
+  <dataValidations count="5">
+    <dataValidation sqref="B3 B4 B5 B6 B7 B8 B9 B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"senior_term,senior_rcf,capex_facility,mezzanine,shl,bond,note,frn,private_placement"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3 C4 C5 C6 C7 C8 C9 C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"loan,bond,note,frn,il_bond,private_placement,convertible"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K3 K4 K5 K6 K7 K8 K9 K10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"fixed,floating,index_linked,hybrid"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M3 M4 M5 M6 M7 M8 M9 M10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"bullet,amortising,sculpted,cash_sweep"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"active,repaid,cancelled,restructured"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17388,7 +18336,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24388,7 +25336,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31388,7 +32336,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31904,305 +32852,6 @@
     </dataValidation>
     <dataValidation sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"C1 - None,C2 - Comfort,C3 - Reserve,C4 - Funded,C5 - Overcollateralised"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CAPITAL STRUCTURE INSTRUMENTS — One row per debt instrument</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Instrument Name</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Security Ranking</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Pari-Passu Group</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Committed Amount</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Drawn Amount</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Margin (bps)</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Base Rate</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Interest Type</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>Maturity Date</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Repayment Type</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Our Holding Amount</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Our Holding %</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>DSRA Months</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="n"/>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="7" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="7" t="n"/>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="n"/>
-      <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="7" t="n"/>
-      <c r="Q3" s="7" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="n"/>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="7" t="n"/>
-      <c r="Q5" s="7" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="7" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
-  </mergeCells>
-  <dataValidations count="5">
-    <dataValidation sqref="B3 B4 B5 B6 B7 B8 B9 B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"senior_term,senior_rcf,capex_facility,mezzanine,shl,bond,note,frn,private_placement"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C3 C4 C5 C6 C7 C8 C9 C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"loan,bond,note,frn,il_bond,private_placement,convertible"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K3 K4 K5 K6 K7 K8 K9 K10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"fixed,floating,index_linked,hybrid"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M3 M4 M5 M6 M7 M8 M9 M10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"bullet,amortising,sculpted,cash_sweep"</formula1>
-    </dataValidation>
-    <dataValidation sqref="Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"active,repaid,cancelled,restructured"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -32909,10 +33558,10 @@
     <dataValidation sqref="B3 B4 B5 B6 B7 B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"opco,bidco,holdco,topco,spv,issuer,guarantor,servicer"</formula1>
     </dataValidation>
-    <dataValidation sqref="B7 B8 B9 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="B7 B8 B9 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -33101,7 +33750,7 @@
     <dataValidation sqref="F3 F4 F5 F6 F7 F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"quarterly,semi_annual,annual"</formula1>
     </dataValidation>
-    <dataValidation sqref="B7 B8 B9 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B81 B87 E3 E4 E5 E6 E7 E8 F3 F4 F5 F6 F7 F8 K3 K4 K5 K6 K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>